<commit_message>
chore: Replace backend and frontend with correct OnboardingModule repositories
- Replaced backend/ with https://github.com/blitzenx25/OnboardingModule-Backend (main branch)
- Replaced frontend/ with https://github.com/blitzenx25/OnboardingModule-Frontend (main branch)
- Removed outdated WROS placeholder code
- Integrated production-ready authentication and UI from source repositories

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/WROS_Canonical_Backlog_S001-401.xlsx
+++ b/backend/WROS_Canonical_Backlog_S001-401.xlsx
@@ -3028,7 +3028,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -6946,7 +6946,7 @@
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P80" s="2" t="inlineStr">
@@ -7026,7 +7026,7 @@
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P81" s="2" t="inlineStr">
@@ -7106,7 +7106,7 @@
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P82" s="2" t="inlineStr">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P83" s="2" t="inlineStr">
@@ -7266,7 +7266,7 @@
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P84" s="2" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr">
@@ -7504,7 +7504,7 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
@@ -7584,7 +7584,7 @@
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P88" s="2" t="inlineStr">
@@ -7664,7 +7664,7 @@
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P89" s="2" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P90" s="2" t="inlineStr">
@@ -7824,7 +7824,7 @@
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P91" s="2" t="inlineStr">
@@ -7904,7 +7904,7 @@
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P92" s="2" t="inlineStr">
@@ -7984,7 +7984,7 @@
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P93" s="2" t="inlineStr">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P94" s="2" t="inlineStr">
@@ -8144,7 +8144,7 @@
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P95" s="2" t="inlineStr">
@@ -8224,7 +8224,7 @@
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P96" s="2" t="inlineStr">
@@ -8304,7 +8304,7 @@
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P97" s="2" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P98" s="2" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P99" s="2" t="inlineStr">
@@ -8544,7 +8544,7 @@
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P100" s="2" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P101" s="2" t="inlineStr">
@@ -8704,7 +8704,7 @@
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P102" s="2" t="inlineStr">
@@ -8864,7 +8864,7 @@
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P104" s="2" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P105" s="2" t="inlineStr">
@@ -9184,7 +9184,7 @@
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P108" s="2" t="inlineStr">
@@ -9264,7 +9264,7 @@
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P109" s="2" t="inlineStr">
@@ -9344,7 +9344,7 @@
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P110" s="2" t="inlineStr">
@@ -9424,7 +9424,7 @@
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P111" s="2" t="inlineStr">
@@ -9504,7 +9504,7 @@
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P112" s="2" t="inlineStr">
@@ -9584,7 +9584,7 @@
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P113" s="2" t="inlineStr">
@@ -9664,7 +9664,7 @@
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P114" s="2" t="inlineStr">
@@ -9744,7 +9744,7 @@
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P115" s="2" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P116" s="2" t="inlineStr">
@@ -9904,7 +9904,7 @@
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P117" s="2" t="inlineStr">
@@ -9984,7 +9984,7 @@
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P118" s="2" t="inlineStr">
@@ -10064,7 +10064,7 @@
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P119" s="2" t="inlineStr">
@@ -10144,7 +10144,7 @@
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P120" s="2" t="inlineStr">
@@ -10224,7 +10224,7 @@
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P121" s="2" t="inlineStr">
@@ -10304,7 +10304,7 @@
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P122" s="2" t="inlineStr">
@@ -10384,7 +10384,7 @@
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P123" s="2" t="inlineStr">
@@ -10464,7 +10464,7 @@
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P124" s="2" t="inlineStr">
@@ -10544,7 +10544,7 @@
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P125" s="2" t="inlineStr">
@@ -10624,7 +10624,7 @@
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P126" s="2" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P127" s="2" t="inlineStr">
@@ -10784,7 +10784,7 @@
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P128" s="2" t="inlineStr">
@@ -10864,7 +10864,7 @@
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P129" s="2" t="inlineStr">
@@ -10944,7 +10944,7 @@
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
@@ -11024,7 +11024,7 @@
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P131" s="2" t="inlineStr">
@@ -11104,7 +11104,7 @@
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P132" s="2" t="inlineStr">
@@ -11184,7 +11184,7 @@
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P133" s="2" t="inlineStr">
@@ -11264,7 +11264,7 @@
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
@@ -11344,7 +11344,7 @@
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P135" s="2" t="inlineStr">
@@ -11424,7 +11424,7 @@
       </c>
       <c r="O136" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P136" s="2" t="inlineStr">
@@ -11504,7 +11504,7 @@
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P137" s="2" t="inlineStr">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
@@ -11664,7 +11664,7 @@
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P139" s="2" t="inlineStr">
@@ -11744,7 +11744,7 @@
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P140" s="2" t="inlineStr">
@@ -11824,7 +11824,7 @@
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P141" s="2" t="inlineStr">
@@ -11904,7 +11904,7 @@
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P142" s="2" t="inlineStr">
@@ -11984,7 +11984,7 @@
       </c>
       <c r="O143" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P143" s="2" t="inlineStr">
@@ -12064,7 +12064,7 @@
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P144" s="2" t="inlineStr">
@@ -12144,7 +12144,7 @@
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P145" s="2" t="inlineStr">
@@ -12224,7 +12224,7 @@
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P146" s="2" t="inlineStr">
@@ -12304,7 +12304,7 @@
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P147" s="2" t="inlineStr">
@@ -12384,7 +12384,7 @@
       </c>
       <c r="O148" s="10" t="inlineStr">
         <is>
-          <t>RETIRED - MERGED — Sub-Vendor Governance Agent (De</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P148" s="10" t="inlineStr">
@@ -12464,7 +12464,7 @@
       </c>
       <c r="O149" s="10" t="inlineStr">
         <is>
-          <t>RETIRED - MERGED — Sub-Vendor Scorecard &amp; Analytic</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P149" s="10" t="inlineStr">
@@ -12624,7 +12624,7 @@
       </c>
       <c r="O151" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P151" s="2" t="inlineStr">
@@ -12784,7 +12784,7 @@
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P153" s="2" t="inlineStr">
@@ -12944,7 +12944,7 @@
       </c>
       <c r="O155" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P155" s="2" t="inlineStr">
@@ -13024,7 +13024,7 @@
       </c>
       <c r="O156" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P156" s="2" t="inlineStr">
@@ -13104,7 +13104,7 @@
       </c>
       <c r="O157" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P157" s="2" t="inlineStr">
@@ -13184,7 +13184,7 @@
       </c>
       <c r="O158" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P158" s="2" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="O159" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P159" s="2" t="inlineStr">
@@ -13344,7 +13344,7 @@
       </c>
       <c r="O160" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P160" s="2" t="inlineStr">
@@ -13424,7 +13424,7 @@
       </c>
       <c r="O161" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P161" s="2" t="inlineStr">
@@ -13504,7 +13504,7 @@
       </c>
       <c r="O162" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P162" s="2" t="inlineStr">
@@ -13584,7 +13584,7 @@
       </c>
       <c r="O163" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P163" s="2" t="inlineStr">
@@ -13664,7 +13664,7 @@
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P164" s="2" t="inlineStr">
@@ -13744,7 +13744,7 @@
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P165" s="2" t="inlineStr">
@@ -13824,7 +13824,7 @@
       </c>
       <c r="O166" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P166" s="2" t="inlineStr">
@@ -13904,7 +13904,7 @@
       </c>
       <c r="O167" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P167" s="2" t="inlineStr">
@@ -13984,7 +13984,7 @@
       </c>
       <c r="O168" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P168" s="2" t="inlineStr">
@@ -14064,7 +14064,7 @@
       </c>
       <c r="O169" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P169" s="2" t="inlineStr">
@@ -14144,7 +14144,7 @@
       </c>
       <c r="O170" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P170" s="2" t="inlineStr">
@@ -14224,7 +14224,7 @@
       </c>
       <c r="O171" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P171" s="2" t="inlineStr">
@@ -14304,7 +14304,7 @@
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P172" s="2" t="inlineStr">
@@ -14384,7 +14384,7 @@
       </c>
       <c r="O173" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P173" s="2" t="inlineStr">
@@ -14464,7 +14464,7 @@
       </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P174" s="2" t="inlineStr">
@@ -14544,7 +14544,7 @@
       </c>
       <c r="O175" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P175" s="2" t="inlineStr">
@@ -14624,7 +14624,7 @@
       </c>
       <c r="O176" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P176" s="2" t="inlineStr">
@@ -14704,7 +14704,7 @@
       </c>
       <c r="O177" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P177" s="2" t="inlineStr">
@@ -14784,7 +14784,7 @@
       </c>
       <c r="O178" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P178" s="2" t="inlineStr">
@@ -14864,7 +14864,7 @@
       </c>
       <c r="O179" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P179" s="2" t="inlineStr">
@@ -14944,7 +14944,7 @@
       </c>
       <c r="O180" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P180" s="2" t="inlineStr">
@@ -15024,7 +15024,7 @@
       </c>
       <c r="O181" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P181" s="2" t="inlineStr">
@@ -15104,7 +15104,7 @@
       </c>
       <c r="O182" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P182" s="2" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="O183" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P183" s="2" t="inlineStr">
@@ -15264,7 +15264,7 @@
       </c>
       <c r="O184" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P184" s="2" t="inlineStr">
@@ -15344,7 +15344,7 @@
       </c>
       <c r="O185" s="10" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P185" s="10" t="inlineStr">
@@ -15584,7 +15584,7 @@
       </c>
       <c r="O188" s="10" t="inlineStr">
         <is>
-          <t>RETIRED - MERGED — RFP Intake, AI Field Extraction</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P188" s="10" t="inlineStr">
@@ -15824,7 +15824,7 @@
       </c>
       <c r="O191" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P191" s="2" t="inlineStr">
@@ -15904,7 +15904,7 @@
       </c>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P192" s="2" t="inlineStr">
@@ -15984,7 +15984,7 @@
       </c>
       <c r="O193" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P193" s="2" t="inlineStr">
@@ -16064,7 +16064,7 @@
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
@@ -16144,7 +16144,7 @@
       </c>
       <c r="O195" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P195" s="2" t="inlineStr">
@@ -16224,7 +16224,7 @@
       </c>
       <c r="O196" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P196" s="2" t="inlineStr">
@@ -16304,7 +16304,7 @@
       </c>
       <c r="O197" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P197" s="2" t="inlineStr">
@@ -16384,7 +16384,7 @@
       </c>
       <c r="O198" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P198" s="2" t="inlineStr">
@@ -16464,7 +16464,7 @@
       </c>
       <c r="O199" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P199" s="2" t="inlineStr">
@@ -18224,7 +18224,7 @@
       </c>
       <c r="O221" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P221" s="2" t="inlineStr">
@@ -18304,7 +18304,7 @@
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P222" s="2" t="inlineStr">
@@ -18384,7 +18384,7 @@
       </c>
       <c r="O223" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P223" s="2" t="inlineStr">
@@ -19024,7 +19024,7 @@
       </c>
       <c r="O231" s="10" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P231" s="10" t="inlineStr">
@@ -19664,7 +19664,7 @@
       </c>
       <c r="O239" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P239" s="2" t="inlineStr">
@@ -19984,7 +19984,7 @@
       </c>
       <c r="O243" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P243" s="2" t="inlineStr">
@@ -20064,7 +20064,7 @@
       </c>
       <c r="O244" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P244" s="2" t="inlineStr">
@@ -21184,7 +21184,7 @@
       </c>
       <c r="O258" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P258" s="2" t="inlineStr">
@@ -21264,7 +21264,7 @@
       </c>
       <c r="O259" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P259" s="2" t="inlineStr">
@@ -21504,7 +21504,7 @@
       </c>
       <c r="O262" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P262" s="2" t="inlineStr">
@@ -21744,7 +21744,7 @@
       </c>
       <c r="O265" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P265" s="2" t="inlineStr">
@@ -21904,7 +21904,7 @@
       </c>
       <c r="O267" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P267" s="2" t="inlineStr">
@@ -22064,7 +22064,7 @@
       </c>
       <c r="O269" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P269" s="2" t="inlineStr">
@@ -22144,7 +22144,7 @@
       </c>
       <c r="O270" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P270" s="2" t="inlineStr">
@@ -22224,7 +22224,7 @@
       </c>
       <c r="O271" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P271" s="2" t="inlineStr">
@@ -22304,7 +22304,7 @@
       </c>
       <c r="O272" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P272" s="2" t="inlineStr">
@@ -22384,7 +22384,7 @@
       </c>
       <c r="O273" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P273" s="2" t="inlineStr">
@@ -22464,7 +22464,7 @@
       </c>
       <c r="O274" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P274" s="2" t="inlineStr">
@@ -22544,7 +22544,7 @@
       </c>
       <c r="O275" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P275" s="2" t="inlineStr">
@@ -22624,7 +22624,7 @@
       </c>
       <c r="O276" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P276" s="2" t="inlineStr">
@@ -22704,7 +22704,7 @@
       </c>
       <c r="O277" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P277" s="2" t="inlineStr">
@@ -22784,7 +22784,7 @@
       </c>
       <c r="O278" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P278" s="2" t="inlineStr">
@@ -22864,7 +22864,7 @@
       </c>
       <c r="O279" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P279" s="2" t="inlineStr">
@@ -22944,7 +22944,7 @@
       </c>
       <c r="O280" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P280" s="2" t="inlineStr">
@@ -23024,7 +23024,7 @@
       </c>
       <c r="O281" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P281" s="2" t="inlineStr">
@@ -23104,7 +23104,7 @@
       </c>
       <c r="O282" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>READY FOR BUILD</t>
         </is>
       </c>
       <c r="P282" s="2" t="inlineStr">
@@ -23184,7 +23184,7 @@
       </c>
       <c r="O283" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P283" s="2" t="inlineStr">
@@ -23264,7 +23264,7 @@
       </c>
       <c r="O284" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P284" s="2" t="inlineStr">
@@ -23344,7 +23344,7 @@
       </c>
       <c r="O285" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P285" s="2" t="inlineStr">
@@ -23424,7 +23424,7 @@
       </c>
       <c r="O286" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P286" s="2" t="inlineStr">
@@ -23504,7 +23504,7 @@
       </c>
       <c r="O287" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P287" s="2" t="inlineStr">
@@ -23584,7 +23584,7 @@
       </c>
       <c r="O288" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P288" s="2" t="inlineStr">
@@ -23664,7 +23664,7 @@
       </c>
       <c r="O289" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P289" s="2" t="inlineStr">
@@ -23744,7 +23744,7 @@
       </c>
       <c r="O290" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P290" s="2" t="inlineStr">
@@ -23824,7 +23824,7 @@
       </c>
       <c r="O291" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P291" s="2" t="inlineStr">
@@ -23904,7 +23904,7 @@
       </c>
       <c r="O292" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P292" s="2" t="inlineStr">
@@ -23984,7 +23984,7 @@
       </c>
       <c r="O293" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P293" s="2" t="inlineStr">
@@ -24064,7 +24064,7 @@
       </c>
       <c r="O294" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P294" s="2" t="inlineStr">
@@ -24144,7 +24144,7 @@
       </c>
       <c r="O295" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P295" s="2" t="inlineStr">
@@ -24304,7 +24304,7 @@
       </c>
       <c r="O297" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P297" s="2" t="inlineStr">
@@ -24384,7 +24384,7 @@
       </c>
       <c r="O298" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P298" s="2" t="inlineStr">
@@ -24464,7 +24464,7 @@
       </c>
       <c r="O299" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P299" s="2" t="inlineStr">
@@ -24544,7 +24544,7 @@
       </c>
       <c r="O300" s="10" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P300" s="10" t="inlineStr">
@@ -24704,7 +24704,7 @@
       </c>
       <c r="O302" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P302" s="2" t="inlineStr">
@@ -24784,7 +24784,7 @@
       </c>
       <c r="O303" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P303" s="2" t="inlineStr">
@@ -24864,7 +24864,7 @@
       </c>
       <c r="O304" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P304" s="2" t="inlineStr">
@@ -24944,7 +24944,7 @@
       </c>
       <c r="O305" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P305" s="2" t="inlineStr">
@@ -25024,7 +25024,7 @@
       </c>
       <c r="O306" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P306" s="2" t="inlineStr">
@@ -25104,7 +25104,7 @@
       </c>
       <c r="O307" s="10" t="inlineStr">
         <is>
-          <t>RETIRED - MERGED — Unified Prediction Engine: Tale</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P307" s="10" t="inlineStr">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="O310" s="10" t="inlineStr">
         <is>
-          <t>RETIRED - MERGED — Unified Prediction Engine: Fina</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P310" s="10" t="inlineStr">
@@ -25504,7 +25504,7 @@
       </c>
       <c r="O312" s="8" t="inlineStr">
         <is>
-          <t>RETIRED — merged into S-309</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P312" s="8" t="inlineStr">
@@ -25584,7 +25584,7 @@
       </c>
       <c r="O313" s="8" t="inlineStr">
         <is>
-          <t>RETIRED — folded into AI Activity Feed / Recruiter Copilot (S-061)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P313" s="8" t="inlineStr">
@@ -25664,7 +25664,7 @@
       </c>
       <c r="O314" s="8" t="inlineStr">
         <is>
-          <t>RETIRED — folded into Auto Create Job from Demand (S-289)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P314" s="8" t="inlineStr">
@@ -25744,7 +25744,7 @@
       </c>
       <c r="O315" s="8" t="inlineStr">
         <is>
-          <t>RETIRED — merged into S-306</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P315" s="8" t="inlineStr">
@@ -26304,7 +26304,7 @@
       </c>
       <c r="O322" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P322" s="2" t="inlineStr">
@@ -26384,7 +26384,7 @@
       </c>
       <c r="O323" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P323" s="2" t="inlineStr">
@@ -26464,7 +26464,7 @@
       </c>
       <c r="O324" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P324" s="2" t="inlineStr">
@@ -26704,7 +26704,7 @@
       </c>
       <c r="O327" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P327" s="2" t="inlineStr">
@@ -26784,7 +26784,7 @@
       </c>
       <c r="O328" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P328" s="2" t="inlineStr">
@@ -26864,7 +26864,7 @@
       </c>
       <c r="O329" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P329" s="2" t="inlineStr">
@@ -26944,7 +26944,7 @@
       </c>
       <c r="O330" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P330" s="2" t="inlineStr">
@@ -27024,7 +27024,7 @@
       </c>
       <c r="O331" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P331" s="2" t="inlineStr">
@@ -27104,7 +27104,7 @@
       </c>
       <c r="O332" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P332" s="2" t="inlineStr">
@@ -27184,7 +27184,7 @@
       </c>
       <c r="O333" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P333" s="2" t="inlineStr">
@@ -27264,7 +27264,7 @@
       </c>
       <c r="O334" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P334" s="2" t="inlineStr">
@@ -27344,7 +27344,7 @@
       </c>
       <c r="O335" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P335" s="2" t="inlineStr">
@@ -27424,7 +27424,7 @@
       </c>
       <c r="O336" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P336" s="2" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="O339" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P339" s="2" t="inlineStr">
@@ -27984,7 +27984,7 @@
       </c>
       <c r="O343" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P343" s="2" t="inlineStr">
@@ -28064,7 +28064,7 @@
       </c>
       <c r="O344" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P344" s="2" t="inlineStr">
@@ -28144,7 +28144,7 @@
       </c>
       <c r="O345" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P345" s="2" t="inlineStr">
@@ -28224,7 +28224,7 @@
       </c>
       <c r="O346" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P346" s="2" t="inlineStr">
@@ -28380,7 +28380,7 @@
       </c>
       <c r="O348" s="2" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>NEW — Ready for Build</t>
         </is>
       </c>
       <c r="P348" s="2" t="inlineStr">
@@ -28770,7 +28770,7 @@
       </c>
       <c r="O353" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P353" s="4" t="inlineStr">
@@ -29004,7 +29004,7 @@
       </c>
       <c r="O356" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P356" s="4" t="inlineStr">
@@ -29160,7 +29160,7 @@
       </c>
       <c r="O358" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P358" s="4" t="inlineStr">
@@ -29862,7 +29862,7 @@
       </c>
       <c r="O367" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P367" s="4" t="inlineStr">
@@ -29940,7 +29940,7 @@
       </c>
       <c r="O368" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P368" s="4" t="inlineStr">
@@ -30018,7 +30018,7 @@
       </c>
       <c r="O369" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P369" s="4" t="inlineStr">
@@ -30096,7 +30096,7 @@
       </c>
       <c r="O370" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P370" s="4" t="inlineStr">
@@ -30174,7 +30174,7 @@
       </c>
       <c r="O371" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P371" s="4" t="inlineStr">
@@ -30252,7 +30252,7 @@
       </c>
       <c r="O372" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P372" s="4" t="inlineStr">
@@ -30486,7 +30486,7 @@
       </c>
       <c r="O375" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P375" s="4" t="inlineStr">
@@ -30564,7 +30564,7 @@
       </c>
       <c r="O376" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P376" s="4" t="inlineStr">
@@ -30642,7 +30642,7 @@
       </c>
       <c r="O377" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P377" s="4" t="inlineStr">
@@ -30720,7 +30720,7 @@
       </c>
       <c r="O378" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P378" s="4" t="inlineStr">
@@ -30798,7 +30798,7 @@
       </c>
       <c r="O379" s="4" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P379" s="4" t="inlineStr">
@@ -30876,7 +30876,7 @@
       </c>
       <c r="O380" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P380" s="12" t="inlineStr">
@@ -30954,7 +30954,7 @@
       </c>
       <c r="O381" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P381" s="12" t="inlineStr">
@@ -31032,7 +31032,7 @@
       </c>
       <c r="O382" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P382" s="12" t="inlineStr">
@@ -31110,7 +31110,7 @@
       </c>
       <c r="O383" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P383" s="12" t="inlineStr">
@@ -31188,7 +31188,7 @@
       </c>
       <c r="O384" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P384" s="12" t="inlineStr">
@@ -31266,7 +31266,7 @@
       </c>
       <c r="O385" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="P385" s="12" t="inlineStr">
@@ -31344,7 +31344,7 @@
       </c>
       <c r="O386" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P386" s="12" t="inlineStr">
@@ -31422,7 +31422,7 @@
       </c>
       <c r="O387" s="12" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P387" s="12" t="inlineStr">
@@ -31734,7 +31734,7 @@
       </c>
       <c r="O391" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P391" s="14" t="inlineStr">
@@ -31812,7 +31812,7 @@
       </c>
       <c r="O392" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P392" s="14" t="inlineStr">
@@ -31890,7 +31890,7 @@
       </c>
       <c r="O393" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P393" s="14" t="inlineStr">
@@ -31968,7 +31968,7 @@
       </c>
       <c r="O394" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P394" s="14" t="inlineStr">
@@ -32046,7 +32046,7 @@
       </c>
       <c r="O395" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P395" s="14" t="inlineStr">
@@ -32124,7 +32124,7 @@
       </c>
       <c r="O396" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P396" s="14" t="inlineStr">
@@ -32202,7 +32202,7 @@
       </c>
       <c r="O397" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P397" s="14" t="inlineStr">
@@ -32280,7 +32280,7 @@
       </c>
       <c r="O398" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P398" s="14" t="inlineStr">
@@ -32358,7 +32358,7 @@
       </c>
       <c r="O399" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P399" s="14" t="inlineStr">
@@ -32436,7 +32436,7 @@
       </c>
       <c r="O400" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P400" s="14" t="inlineStr">
@@ -32514,7 +32514,7 @@
       </c>
       <c r="O401" s="14" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Ready for Build</t>
         </is>
       </c>
       <c r="P401" s="14" t="inlineStr">
@@ -32594,7 +32594,7 @@
       </c>
       <c r="O402" s="14" t="inlineStr">
         <is>
-          <t>BLOCKED — Awaiting Finance/CA Requirements Review</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="P402" s="14" t="inlineStr">
@@ -32789,7 +32789,7 @@
       </c>
       <c r="O405" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P405" t="inlineStr">
@@ -32854,7 +32854,7 @@
       </c>
       <c r="O406" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P406" t="inlineStr">
@@ -32919,7 +32919,7 @@
       </c>
       <c r="O407" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P407" t="inlineStr">
@@ -32984,7 +32984,7 @@
       </c>
       <c r="O408" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P408" t="inlineStr">
@@ -33049,7 +33049,7 @@
       </c>
       <c r="O409" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P409" t="inlineStr">
@@ -33114,7 +33114,7 @@
       </c>
       <c r="O410" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P410" t="inlineStr">
@@ -33179,7 +33179,7 @@
       </c>
       <c r="O411" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P411" t="inlineStr">
@@ -33244,7 +33244,7 @@
       </c>
       <c r="O412" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P412" t="inlineStr">
@@ -33309,7 +33309,7 @@
       </c>
       <c r="O413" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P413" t="inlineStr">
@@ -33374,7 +33374,7 @@
       </c>
       <c r="O414" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P414" t="inlineStr">
@@ -33439,7 +33439,7 @@
       </c>
       <c r="O415" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P415" t="inlineStr">
@@ -33504,7 +33504,7 @@
       </c>
       <c r="O416" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P416" t="inlineStr">
@@ -33569,7 +33569,7 @@
       </c>
       <c r="O417" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P417" t="inlineStr">
@@ -33634,7 +33634,7 @@
       </c>
       <c r="O418" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P418" t="inlineStr">
@@ -33699,7 +33699,7 @@
       </c>
       <c r="O419" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P419" t="inlineStr">
@@ -33764,7 +33764,7 @@
       </c>
       <c r="O420" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P420" t="inlineStr">
@@ -33829,7 +33829,7 @@
       </c>
       <c r="O421" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P421" t="inlineStr">
@@ -33894,7 +33894,7 @@
       </c>
       <c r="O422" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P422" t="inlineStr">
@@ -33959,7 +33959,7 @@
       </c>
       <c r="O423" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P423" t="inlineStr">
@@ -34024,7 +34024,7 @@
       </c>
       <c r="O424" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P424" t="inlineStr">
@@ -34089,7 +34089,7 @@
       </c>
       <c r="O425" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P425" t="inlineStr">
@@ -34154,7 +34154,7 @@
       </c>
       <c r="O426" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P426" t="inlineStr">
@@ -34219,7 +34219,7 @@
       </c>
       <c r="O427" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P427" t="inlineStr">
@@ -34284,7 +34284,7 @@
       </c>
       <c r="O428" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P428" t="inlineStr">
@@ -34349,7 +34349,7 @@
       </c>
       <c r="O429" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P429" t="inlineStr">
@@ -34414,7 +34414,7 @@
       </c>
       <c r="O430" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P430" t="inlineStr">
@@ -34479,7 +34479,7 @@
       </c>
       <c r="O431" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P431" t="inlineStr">
@@ -34544,7 +34544,7 @@
       </c>
       <c r="O432" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P432" t="inlineStr">
@@ -34609,7 +34609,7 @@
       </c>
       <c r="O433" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P433" t="inlineStr">
@@ -34674,7 +34674,7 @@
       </c>
       <c r="O434" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Planned</t>
         </is>
       </c>
       <c r="P434" t="inlineStr">

</xml_diff>